<commit_message>
Use the quotation letterhead as the header in the generated PO Excel
</commit_message>
<xml_diff>
--- a/public/templates/po-2307-template.xlsx
+++ b/public/templates/po-2307-template.xlsx
@@ -3100,19 +3100,14 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>121677</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>36928</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>597218</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>36928</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="6667500" cy="1638300"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -3143,183 +3138,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>246772</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>16168</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>172477</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>16168</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>91109</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>57978</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>495932</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>71510</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>102453</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>473848</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>442278</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>157779</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>190149</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>29920</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>157407</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>10889</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3723,7 +3542,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD84"/>
+  <dimension ref="A11:AD84"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
@@ -3739,16 +3558,6 @@
     <col min="28" max="28" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25"/>
     <row r="11" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J11" s="4"/>
     </row>
@@ -3884,7 +3693,7 @@
       <c r="I20" s="23"/>
       <c r="J20" s="24"/>
     </row>
-    <row r="21" ht="22.5" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" ht="22.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="25" t="s">
         <v>12</v>
       </c>
@@ -3902,7 +3711,7 @@
       <c r="M21" s="1"/>
       <c r="N21" s="30"/>
     </row>
-    <row r="22" ht="22.5" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" ht="22.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
         <v>13</v>
       </c>
@@ -3919,7 +3728,7 @@
       <c r="M22" s="32"/>
       <c r="N22" s="30"/>
     </row>
-    <row r="23" ht="23.25" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" ht="23.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
         <v>14</v>
       </c>
@@ -3935,7 +3744,7 @@
       <c r="M23" s="1"/>
       <c r="N23" s="30"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" ht="16.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="33" t="s">
         <v>15</v>
       </c>
@@ -4099,7 +3908,7 @@
       <c r="I44" s="17"/>
       <c r="J44" s="17"/>
     </row>
-    <row r="45" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" ht="45" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="21"/>
       <c r="B45" s="54"/>
       <c r="C45" s="1"/>
@@ -4110,7 +3919,7 @@
       <c r="I45" s="23"/>
       <c r="J45" s="24"/>
     </row>
-    <row r="46" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" ht="45" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="21"/>
       <c r="B46" s="54"/>
       <c r="C46" s="1"/>
@@ -4121,7 +3930,7 @@
       <c r="I46" s="23"/>
       <c r="J46" s="24"/>
     </row>
-    <row r="47" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" ht="45" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="21"/>
       <c r="B47" s="54"/>
       <c r="C47" s="1"/>
@@ -4144,7 +3953,7 @@
       <c r="I48" s="59"/>
       <c r="J48" s="60"/>
     </row>
-    <row r="59" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C59" s="1"/>
       <c r="D59" s="2"/>
       <c r="F59" s="1"/>
@@ -4153,7 +3962,7 @@
       <c r="I59" s="1"/>
       <c r="J59" s="3"/>
     </row>
-    <row r="63" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C63" s="1"/>
       <c r="D63" s="2"/>
       <c r="F63" s="1"/>
@@ -4164,7 +3973,7 @@
       <c r="AB63" s="61"/>
       <c r="AD63" s="29"/>
     </row>
-    <row r="64" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C64" s="1"/>
       <c r="D64" s="2"/>
       <c r="F64" s="1"/>
@@ -4175,7 +3984,7 @@
       <c r="AB64" s="62"/>
       <c r="AD64" s="29"/>
     </row>
-    <row r="65" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C65" s="1"/>
       <c r="D65" s="2"/>
       <c r="F65" s="1"/>
@@ -4186,7 +3995,7 @@
       <c r="AB65" s="61"/>
       <c r="AD65" s="29"/>
     </row>
-    <row r="66" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C66" s="1"/>
       <c r="D66" s="2"/>
       <c r="F66" s="1"/>
@@ -4197,7 +4006,7 @@
       <c r="AB66" s="62"/>
       <c r="AD66" s="29"/>
     </row>
-    <row r="67" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C67" s="1"/>
       <c r="D67" s="2"/>
       <c r="F67" s="1"/>
@@ -4208,7 +4017,7 @@
       <c r="AB67" s="61"/>
       <c r="AD67" s="29"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C68" s="1"/>
       <c r="D68" s="2"/>
       <c r="F68" s="1"/>
@@ -4219,7 +4028,7 @@
       <c r="AB68" s="62"/>
       <c r="AD68" s="29"/>
     </row>
-    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C69" s="1"/>
       <c r="D69" s="2"/>
       <c r="F69" s="1"/>
@@ -4230,7 +4039,7 @@
       <c r="AB69" s="61"/>
       <c r="AD69" s="29"/>
     </row>
-    <row r="70" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C70" s="1"/>
       <c r="D70" s="2"/>
       <c r="F70" s="1"/>
@@ -4241,7 +4050,7 @@
       <c r="AB70" s="62"/>
       <c r="AD70" s="29"/>
     </row>
-    <row r="71" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C71" s="1"/>
       <c r="D71" s="2"/>
       <c r="F71" s="1"/>
@@ -4252,7 +4061,7 @@
       <c r="AB71" s="61"/>
       <c r="AD71" s="29"/>
     </row>
-    <row r="72" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" spans="3:30" x14ac:dyDescent="0.25">
       <c r="C72" s="1"/>
       <c r="D72" s="2"/>
       <c r="F72" s="1"/>
@@ -4263,7 +4072,7 @@
       <c r="AB72" s="62"/>
       <c r="AD72" s="29"/>
     </row>
-    <row r="73" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="73" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C73" s="1"/>
       <c r="D73" s="2"/>
       <c r="F73" s="1"/>
@@ -4273,7 +4082,7 @@
       <c r="J73" s="3"/>
       <c r="AB73" s="61"/>
     </row>
-    <row r="74" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="74" spans="3:28" x14ac:dyDescent="0.25">
       <c r="C74" s="1"/>
       <c r="D74" s="2"/>
       <c r="F74" s="1"/>
@@ -4283,7 +4092,7 @@
       <c r="J74" s="3"/>
       <c r="AB74" s="62"/>
     </row>
-    <row r="77" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="77" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C77" s="1"/>
       <c r="D77" s="2"/>
       <c r="F77" s="1"/>
@@ -4292,7 +4101,7 @@
       <c r="I77" s="1"/>
       <c r="J77" s="3"/>
     </row>
-    <row r="78" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C78" s="1"/>
       <c r="D78" s="2"/>
       <c r="F78" s="1"/>
@@ -4301,7 +4110,7 @@
       <c r="I78" s="1"/>
       <c r="J78" s="3"/>
     </row>
-    <row r="79" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="79" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C79" s="1"/>
       <c r="D79" s="2"/>
       <c r="F79" s="1"/>
@@ -4310,7 +4119,7 @@
       <c r="I79" s="1"/>
       <c r="J79" s="3"/>
     </row>
-    <row r="80" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="80" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C80" s="1"/>
       <c r="D80" s="2"/>
       <c r="F80" s="1"/>
@@ -4319,7 +4128,7 @@
       <c r="I80" s="1"/>
       <c r="J80" s="3"/>
     </row>
-    <row r="81" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="81" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C81" s="1"/>
       <c r="D81" s="2"/>
       <c r="F81" s="1"/>
@@ -4328,7 +4137,7 @@
       <c r="I81" s="1"/>
       <c r="J81" s="3"/>
     </row>
-    <row r="82" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="82" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C82" s="1"/>
       <c r="D82" s="2"/>
       <c r="F82" s="1"/>
@@ -4337,7 +4146,7 @@
       <c r="I82" s="1"/>
       <c r="J82" s="3"/>
     </row>
-    <row r="83" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C83" s="1"/>
       <c r="D83" s="2"/>
       <c r="F83" s="1"/>
@@ -4346,7 +4155,7 @@
       <c r="I83" s="1"/>
       <c r="J83" s="3"/>
     </row>
-    <row r="84" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="84" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C84" s="1"/>
       <c r="D84" s="2"/>
       <c r="F84" s="1"/>

</xml_diff>